<commit_message>
Revise Bill of Exchange Q&A: drop savings/FTE figures, bold TBC for unknowns
- Remove all monetary savings amounts and FTE numbers from the
  responses (Solution/KPI rows in particular), keeping the answers
  qualitative
- Replace speculative specifics not found in the Business Case or PQD
  (e.g. exact form fields, mandatory attachments, headcounts) with a
  bold TBC so the SME can complete them on review

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T3ELd5gwFVvkXx8ntq4vH7
</commit_message>
<xml_diff>
--- a/UST_QA_Bill_of_Exchange.xlsx
+++ b/UST_QA_Bill_of_Exchange.xlsx
@@ -577,7 +577,7 @@
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>All of the above. The platform tackles efficiency (removing manual, Outlook-based handling of bills of exchange and cheques, reducing effort from ~0.58 to ~0.01 FTE), standardization (a single centralized platform for requesting, approving and posting, replacing dispersed email requests), compliance (full alignment with SODA authorization and SOX controls) and auditability (systematic retention of process evidence for internal audits). Reducing data and human errors is a further driver.</t>
+          <t>All of the above. The platform tackles efficiency (removing the manual, Outlook-based handling of bills of exchange and cheques and cutting manual workload), standardization (a single centralized platform for requesting, approving and posting, replacing dispersed email requests), compliance (full alignment with SODA authorization and SOX controls) and auditability (systematic retention of process evidence for internal audits). Reducing data and human errors is a further driver.</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Measured against the AS-IS vs TO-BE business case: reduction in manual effort/FTE (0.58 -&gt; 0.01 FTE), annual cost saving (~EUR 23k), share of the process automated (~90%), reduction in data/human errors, elimination of the manual Outlook workload, and 100% availability of SODA/SOX audit evidence. Meeting bank posting deadlines with continuous/daily posting is also a success measure.</t>
+          <t>Measured against the AS-IS vs TO-BE business case: reduced manual effort, lower operating cost, a high share of the process automated, fewer data/human errors, elimination of the manual Outlook workload, and 100% availability of SODA/SOX audit evidence. Meeting bank posting deadlines with continuous/daily posting is also a success measure.</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Target KPIs: FTE saving ~0.57 (from 0.58 to 0.01), ~98% reduction in manual effort; annual cost saving ~EUR 23,090; ~90% of the process automated; manual processing time reduced from ~7 min/transaction toward near-zero; measurable reduction in data/human errors; 100% SODA/SOX compliance and audit-evidence retention. Expected business impact is rated 5/5 for error reduction, efficiency and standardization/compliance.</t>
+          <t>Target KPIs: a significant reduction in manual effort and in manual processing time per transaction (currently ~7 minutes), ~90% of the process automated, a measurable reduction in data/human errors, and 100% SODA/SOX compliance with full audit-evidence retention. Expected business impact is rated 5/5 for error reduction, efficiency and standardization/compliance.</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,28 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>AS-IS volumes are ~455 bills of exchange and ~178 cheques per month (~633 items/month), i.e. roughly 30-36 items per working day on average (PQD: ~36 cases per daily run). Peaks occur around bank posting cut-offs and month-end. Precise peak-day figures to be confirmed with the Banking team.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">AS-IS volumes are ~455 bills of exchange and ~178 cheques per month (~633 items/month), i.e. roughly 30-36 items per working day on average. Peaks occur around bank posting cut-offs and month-end. Precise peak-day figures are </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -659,7 +680,28 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Yes - bills of exchange and cheques cluster around their due dates and bank posting deadlines, so volumes concentrate around bank cut-offs and month-end closing. Banking posting deadlines are a defined SLA and posting is expected to be continuous/daily. The detailed spike profile to be confirmed with the Banking team.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Yes - bills of exchange and cheques cluster around their due dates and bank posting deadlines, so volumes concentrate around bank cut-offs and month-end closing. Banking posting deadlines are a defined SLA and posting is expected to be continuous/daily. The detailed spike profile is </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -676,7 +718,21 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>To be finalized in the design workshop. Indicatively, each bill-of-exchange/cheque request is expected to capture: payer/customer, document/reference number, instrument type (bill of exchange or cheque), amount and currency, issue and due dates, bank/account details, company code (SAP E01), posting date, and the linked supporting document. Definitive mandatory-field list TBC.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> - the specific fields required on each request/transaction are not defined in the Business Case or PQD; to be confirmed with the relevant SME.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -702,7 +758,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Not within the current scope: the perimeter is a single country (Morocco region), single ERP (SAP E01) and single division (Iberia SSC - Banking), so there is no cross-country/ERP field variation to accommodate. Mandatory fields will be standardized on the single platform. Variation would only arise if scope is later extended.</t>
+          <t>Not within the current scope: the perimeter is a single country (Morocco region), single ERP (SAP E01) and single division (Iberia SSC - Banking), so there is no cross-country/ERP field variation to accommodate. Mandatory fields will be standardized on the single platform.</t>
         </is>
       </c>
     </row>
@@ -715,7 +771,28 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Each request must carry its supporting evidence - principally the bill-of-exchange/cheque document (image/scan) and any associated banking/supporting document - so that complete evidence is retained per request for internal audit and SOX. The definitive mandatory-attachment list to be confirmed in design.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Supporting evidence must be retained for each request so that a complete audit trail is available for SOX/SODA and internal audit. The specific mandatory documents to attach are </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -728,7 +805,28 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>At business level, before posting the platform must confirm: mandatory-field completeness/validity, credit-management validation, that the request carries the required SODA approval, and correct approval routing (plus duplicate/amount checks to be assessed). Detailed validation rules to be defined in the design phase.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Before posting, the request must pass credit-management validation and carry the required SODA approval. The full set of detailed validation rules is </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -741,7 +839,28 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>The main business exceptions are unpaid bills of exchange (~10% of BoE) and unpaid cheques (~5%), which require dedicated handling. Other exceptions include requests denied at approval, missing/invalid data, and failed credit-management validation. Detailed exception handling to be defined in design.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">The main business exceptions are unpaid bills of exchange (~10% of BoE) and unpaid cheques (~5%), which require dedicated handling. The full list of exception scenarios is </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -771,7 +890,28 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Currently Outlook/email (a shared mailbox) and Excel; banking platforms/portals are used for bill-of-exchange and cheque handling. Process evidence will be retained on the new platform. Specific banking-portal / document-repository names to be confirmed with the Banking team.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Currently Outlook/email (a shared mailbox) and Excel. Banking platforms/portals are also involved in bill-of-exchange and cheque handling; the specific portal / document-repository names are </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -853,7 +993,28 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Evidence supporting SODA authorization and SOX controls must be retained: the request and its data, the approval trail, the supporting bill-of-exchange/cheque document, and the posting confirmation - i.e. full process evidence available for internal audit. Commercially sensitive and GDPR-governed data is involved, so retention must respect GDPR.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Evidence supporting SODA authorization and SOX controls must be retained, together with the complete process trail available for internal audit. Commercially sensitive and GDPR-governed data is involved, so retention must respect GDPR. The specific evidence items and retention periods are </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -866,7 +1027,28 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Reporting is expected on processed volumes (bills of exchange/cheques), unpaid BoE/cheque rates, exception counts, processing time / FTE saving, and compliance/evidence completeness. Specific dashboard layouts and recipients to be confirmed with the Banking team and process owner.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Specific reporting and dashboard requirements are not defined in the Business Case or PQD and are </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (they would logically cover processed volumes, exceptions and compliance evidence).</t>
+          </r>
         </is>
       </c>
     </row>
@@ -883,7 +1065,28 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>To be confirmed. Requestors are the Iberia SSC Banking team members who currently raise bill-of-exchange/cheque requests; the exact headcount will be provided by the process owner (Francisco Manzanilla) / Banking team.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Requestors are the Iberia SSC Banking team members who currently raise bill-of-exchange/cheque requests; the exact number is </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -896,7 +1099,28 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>To be confirmed. Approvers are defined by the SODA authorization matrix for Banking (e.g. team lead / authorized approvers); the exact number will be provided by the process owner / Banking team.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Approvers are defined by the SODA authorization matrix for Banking; the exact number is </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -909,7 +1133,28 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Approval routing is driven by the SODA (segregation-of-duties) authorization matrix / financial authorization levels. Roles are role-based (Requestor vs Approver) mapped to the Iberia SSC Banking team. The detailed role-to-approver mapping will be provided from the SODA matrix.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Approval routing is driven by the SODA (segregation-of-duties) authorization matrix / financial authorization levels, with role-based Requestor vs Approver roles mapped to the Iberia SSC Banking team. The detailed role-to-approver mapping is </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -935,7 +1180,28 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Approval levels follow the SODA financial-authorization thresholds. In principle a request is approved when its data is valid, credit-management validation passes and it is within the approver's authority; it is denied on failed validation/credit checks, missing evidence or policy breach. The detailed approval matrix and thresholds to be provided from the SODA documentation.</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Approval levels follow the SODA financial-authorization thresholds: a request is approved when its data is valid, credit-management validation passes and it is within the approver's authority, and denied on failed validation/credit checks, missing evidence or policy breach. The detailed approval matrix and thresholds are </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TBC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <sz val="11"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Leave technical questions blank in Bill of Exchange Q&A
Clear the responses for the technical/integration questions (rows
19-21: ERP APIs, RPA/Power Automate Desktop, real-time integration) so
they are left blank rather than deferred with text, per request to not
reply to any technical questions.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T3ELd5gwFVvkXx8ntq4vH7
</commit_message>
<xml_diff>
--- a/UST_QA_Bill_of_Exchange.xlsx
+++ b/UST_QA_Bill_of_Exchange.xlsx
@@ -948,11 +948,7 @@
           <t>Are APIs available for each ERP that is in scope</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Technical / integration question - to be addressed by DS Smith IT together with UST Solution Architecture (out of scope for this business response).</t>
-        </is>
-      </c>
+      <c r="C19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -961,11 +957,7 @@
           <t xml:space="preserve"> where API is not available, have you already identified which ERP interactions would require Power Automate Desktop (RPA)?</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Technical / integration question - to be addressed by DS Smith IT together with UST Solution Architecture (out of scope for this business response).</t>
-        </is>
-      </c>
+      <c r="C20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n"/>
@@ -974,11 +966,7 @@
           <t>Is real-time integration required for any of these use case?</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Technical / integration question - to be addressed by DS Smith IT together with UST Solution Architecture (out of scope for this business response).</t>
-        </is>
-      </c>
+      <c r="C21" s="3" t="n"/>
     </row>
     <row r="22" ht="27" customHeight="1">
       <c r="A22" s="4" t="inlineStr">

</xml_diff>